<commit_message>
Update Amazon report + model files (Jul 2026)
</commit_message>
<xml_diff>
--- a/assets/files/amazon-financial-model.xlsx
+++ b/assets/files/amazon-financial-model.xlsx
@@ -809,7 +809,7 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF232F3E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
@@ -1734,7 +1734,7 @@
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -1743,7 +1743,7 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF232F3E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
@@ -2797,7 +2797,7 @@
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -2806,7 +2806,7 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF232F3E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
@@ -3720,7 +3720,7 @@
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -3729,7 +3729,7 @@
   <sheetPr>
     <tabColor rgb="00232F3E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3750,7 +3750,7 @@
     <row r="2">
       <c r="A2" s="63" t="inlineStr">
         <is>
-          <t>Researched Jun 2026 · update with live data before use</t>
+          <t>Researched 10 Jul 2026 · prices as of 9-Jul-2026 close</t>
         </is>
       </c>
     </row>
@@ -3783,10 +3783,10 @@
         </is>
       </c>
       <c r="B5" s="67" t="n">
-        <v>241.7</v>
+        <v>247.04</v>
       </c>
       <c r="C5" s="67" t="n">
-        <v>8.49</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="D5" s="68">
         <f>B5/C5</f>
@@ -3800,7 +3800,7 @@
         </is>
       </c>
       <c r="B6" s="70" t="n">
-        <v>373.02</v>
+        <v>384.25</v>
       </c>
       <c r="C6" s="70" t="n">
         <v>16.86</v>
@@ -3817,7 +3817,7 @@
         </is>
       </c>
       <c r="B7" s="73" t="n">
-        <v>357.37</v>
+        <v>357.24</v>
       </c>
       <c r="C7" s="73" t="n">
         <v>13.24</v>
@@ -3834,7 +3834,7 @@
         </is>
       </c>
       <c r="B8" s="70" t="n">
-        <v>550.25</v>
+        <v>615.6</v>
       </c>
       <c r="C8" s="70" t="n">
         <v>27.95</v>
@@ -3915,5 +3915,6 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh all 11 research notes + models (multi-method rebuild)
Multi-method rebuild: refresh all 11 research notes + models (PDF/xlsx)
</commit_message>
<xml_diff>
--- a/assets/files/amazon-financial-model.xlsx
+++ b/assets/files/amazon-financial-model.xlsx
@@ -7,12 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer Comps" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer Comps" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'SOTP'!$A$1:$F$20</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
@@ -24,7 +27,7 @@
     <numFmt numFmtId="165" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -150,8 +153,13 @@
       <color rgb="00595959"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -196,6 +204,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEF2F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E5496"/>
       </patternFill>
     </fill>
   </fills>
@@ -350,7 +368,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -557,6 +575,11 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -806,6 +829,273 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="30" min="1" max="1"/>
+    <col width="20" customWidth="1" style="30" min="2" max="2"/>
+    <col width="13" customWidth="1" style="30" min="3" max="3"/>
+    <col width="13" customWidth="1" style="30" min="4" max="4"/>
+    <col width="13" customWidth="1" style="30" min="5" max="5"/>
+    <col width="52" customWidth="1" style="30" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="80" t="inlineStr">
+        <is>
+          <t>Amazon.com (AMZN) — Sum-of-the-Parts (SOTP) Valuation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>USD millions except per share. FY2025 segment basis. 10,700M shares; net cash ~$45bn. Live $248 (Jul 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="81" t="inlineStr">
+        <is>
+          <t>SEGMENT VALUATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="B6" s="82" t="inlineStr">
+        <is>
+          <t>Metric (FY25, $M)</t>
+        </is>
+      </c>
+      <c r="C6" s="82" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D6" s="82" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="E6" s="82" t="inlineStr">
+        <is>
+          <t>EV / Value ($M)</t>
+        </is>
+      </c>
+      <c r="F6" s="82" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>128700</v>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="83">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>Crown jewel: +20-24%, ~37% margin, AI tailwind @ 15x rev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Advertising</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>63000</v>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="83">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>+22%, ~50% margin, hidden inside retail @ 8x rev</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>Retail (NA+Intl, ex-ads)</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>588000</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E9" s="83">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>Low-margin e-commerce + logistics moat @ 0.6x rev</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>Net cash</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Cash − debt</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="83">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="29" t="inlineStr">
+        <is>
+          <t>Balance sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="81" t="inlineStr">
+        <is>
+          <t>SOTP SUMMARY &amp; RATING</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Sum of segment values ($M)</t>
+        </is>
+      </c>
+      <c r="B13" s="83">
+        <f>SUM(E7:E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Diluted shares (M)</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n">
+        <v>10700</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>SOTP value per share ($)</t>
+        </is>
+      </c>
+      <c r="B15" s="83">
+        <f>B13/B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>Current price ($)</t>
+        </is>
+      </c>
+      <c r="B16" s="83" t="n">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>Upside / (downside)</t>
+        </is>
+      </c>
+      <c r="B17" s="84">
+        <f>B15/B16-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="B18" s="29">
+        <f>IF(B17&gt;0.10,"BUY",IF(B17&gt;0.03,"ACCUMULATE",IF(B17&gt;-0.08,"HOLD","REDUCE")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Note: AWS is the value engine — SOTP prices it as the standalone hyperscaler the blended multiple hides. Advertising (~$63bn, ~50% margin) is a high-value business buried in retail. Retail carries the moat but thin margins. FCF is temporarily suppressed by ~$200bn AI/logistics capex.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A4:F4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="FF232F3E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1738,7 +2028,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="FF232F3E"/>
@@ -2801,7 +3091,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="FF232F3E"/>
@@ -3724,7 +4014,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00232F3E"/>

</xml_diff>